<commit_message>
Replace Table S2, Table S3 and Figure S15 data and code with the four-condition batch (adds context-only)
Context-only (no data; softened prompt) is added as a fourth condition of the ablation:
prompts, 36 attempts + 12 selected answers, verdicts, quality scorecards (two passes), agreement
records, generation code. Table S2 (generation rates), Table S3 (model-level quality scores) and
Figure S15 (radar, all axes and all conditions first; applicable-axes variant) are regenerated
from the repository data with new folders TableS2_generation_rate/ and TableS3_quality_by_model/.
The displayed criterion name is "Hypothesis Specificity" everywhere. READMEs of the repository,
1_generation_code, 2_prompts, 3_answers, 4_evaluation_code, 5_evaluation_results and
6_supplementary_figures document the new layout.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/5_evaluation_results/ablation_conditions/1_success_rate_table/success_rate_table.xlsx
+++ b/5_evaluation_results/ablation_conditions/1_success_rate_table/success_rate_table.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -535,6 +535,33 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Context-only</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>100% (70-100%)  [9/9]</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>100% (70-100%)  [9/9]</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>100% (70-100%)  [9/9]</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>89% (56-98%)  [8/9]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -546,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -664,6 +691,33 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Context-only</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>9 (incl. 1 with no text at the output cap)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -675,7 +729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -721,7 +775,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -747,7 +801,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -773,7 +827,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -790,16 +844,16 @@
         <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -825,7 +879,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -851,7 +905,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -877,7 +931,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -891,19 +945,19 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F8" t="n">
-        <v>3.3</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -917,19 +971,19 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
         <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>42.9</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -943,19 +997,19 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10" t="n">
         <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -981,7 +1035,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1007,7 +1061,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1033,7 +1087,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1050,16 +1104,16 @@
         <v>3</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1076,16 +1130,16 @@
         <v>3</v>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66.7</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1102,16 +1156,16 @@
         <v>3</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1137,7 +1191,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1163,7 +1217,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1189,7 +1243,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1203,19 +1257,19 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1229,19 +1283,19 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>42.9</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1255,19 +1309,19 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F22" t="n">
-        <v>33.3</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1284,16 +1338,16 @@
         <v>3</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F23" t="n">
-        <v>33.3</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1319,7 +1373,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1336,16 +1390,16 @@
         <v>3</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1362,16 +1416,16 @@
         <v>3</v>
       </c>
       <c r="E26" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1388,16 +1442,16 @@
         <v>3</v>
       </c>
       <c r="E27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F27" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1414,16 +1468,16 @@
         <v>3</v>
       </c>
       <c r="E28" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1449,7 +1503,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1475,7 +1529,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1501,7 +1555,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1518,16 +1572,16 @@
         <v>3</v>
       </c>
       <c r="E32" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1544,16 +1598,16 @@
         <v>3</v>
       </c>
       <c r="E33" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1570,16 +1624,16 @@
         <v>3</v>
       </c>
       <c r="E34" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>100</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1596,16 +1650,16 @@
         <v>3</v>
       </c>
       <c r="E35" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>100</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1631,26 +1685,338 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>Measurement-only</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Gouwens input resistance</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>3</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>PITCH</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>DeepSeek V4.1 Flash</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>CITE-seq CD45RA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>3</v>
+      </c>
+      <c r="E38" t="n">
+        <v>3</v>
+      </c>
+      <c r="F38" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>DeepSeek V4.1 Flash</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>CosMx Ki-67</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>3</v>
+      </c>
+      <c r="E39" t="n">
+        <v>3</v>
+      </c>
+      <c r="F39" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>DeepSeek V4.1 Flash</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Gouwens input resistance</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>3</v>
+      </c>
+      <c r="E40" t="n">
+        <v>3</v>
+      </c>
+      <c r="F40" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>GLM-5.3</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>CITE-seq CD45RA</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" t="n">
+        <v>3</v>
+      </c>
+      <c r="F41" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>GLM-5.3</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>CosMx Ki-67</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>3</v>
+      </c>
+      <c r="E42" t="n">
+        <v>3</v>
+      </c>
+      <c r="F42" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>GLM-5.3</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Gouwens input resistance</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>3</v>
+      </c>
+      <c r="E43" t="n">
+        <v>3</v>
+      </c>
+      <c r="F43" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Gemini-3.1-pro-preview</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>CITE-seq CD45RA</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>3</v>
+      </c>
+      <c r="E44" t="n">
+        <v>3</v>
+      </c>
+      <c r="F44" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Gemini-3.1-pro-preview</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>CosMx Ki-67</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>3</v>
+      </c>
+      <c r="E45" t="n">
+        <v>3</v>
+      </c>
+      <c r="F45" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Gemini-3.1-pro-preview</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Gouwens input resistance</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>3</v>
+      </c>
+      <c r="E46" t="n">
+        <v>3</v>
+      </c>
+      <c r="F46" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
         <is>
           <t>Qwen3.8-2.4T-A95B</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>CITE-seq CD45RA</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>3</v>
+      </c>
+      <c r="E47" t="n">
+        <v>3</v>
+      </c>
+      <c r="F47" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>CosMx Ki-67</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" t="n">
+        <v>3</v>
+      </c>
+      <c r="F48" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
         <is>
           <t>Gouwens input resistance</t>
         </is>
       </c>
-      <c r="D37" t="n">
-        <v>3</v>
-      </c>
-      <c r="E37" t="n">
-        <v>3</v>
-      </c>
-      <c r="F37" t="n">
+      <c r="D49" t="n">
+        <v>3</v>
+      </c>
+      <c r="E49" t="n">
+        <v>3</v>
+      </c>
+      <c r="F49" t="n">
         <v>100</v>
       </c>
     </row>
@@ -1665,7 +2031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F141"/>
+  <dimension ref="A1:F177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1716,7 +2082,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1744,7 +2110,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1772,7 +2138,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1800,7 +2166,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1828,7 +2194,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1856,7 +2222,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1884,7 +2250,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1912,7 +2278,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1925,11 +2291,11 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>no text (hit output cap)</t>
         </is>
       </c>
       <c r="F9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1940,7 +2306,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1968,7 +2334,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1981,11 +2347,11 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>no text (hit output cap)</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -1996,7 +2362,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2009,11 +2375,11 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -2024,7 +2390,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2037,11 +2403,11 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -2052,7 +2418,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2080,7 +2446,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2108,7 +2474,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2121,11 +2487,11 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -2136,7 +2502,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2149,11 +2515,11 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>no text (hit output cap)</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -2164,7 +2530,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2177,11 +2543,11 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -2192,7 +2558,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2205,11 +2571,11 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -2220,7 +2586,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2233,11 +2599,11 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>no text (hit output cap)</t>
         </is>
       </c>
       <c r="F20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -2248,7 +2614,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2261,11 +2627,11 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -2276,7 +2642,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2289,11 +2655,11 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -2304,7 +2670,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2332,7 +2698,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2360,7 +2726,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2373,11 +2739,11 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="F25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -2388,7 +2754,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2401,11 +2767,11 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>no text (hit output cap)</t>
         </is>
       </c>
       <c r="F26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -2416,7 +2782,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2429,11 +2795,11 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -2444,7 +2810,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2457,22 +2823,22 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>GLM-5.3</t>
+          <t>DeepSeek V4.1 Flash</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>PITCH</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2495,12 +2861,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>GLM-5.3</t>
+          <t>DeepSeek V4.1 Flash</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>PITCH</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2523,12 +2889,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>GLM-5.3</t>
+          <t>DeepSeek V4.1 Flash</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>PITCH</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2551,12 +2917,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GLM-5.3</t>
+          <t>DeepSeek V4.1 Flash</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>PITCH</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2579,12 +2945,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>GLM-5.3</t>
+          <t>DeepSeek V4.1 Flash</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>PITCH</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2607,12 +2973,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>GLM-5.3</t>
+          <t>DeepSeek V4.1 Flash</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>PITCH</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2635,12 +3001,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>GLM-5.3</t>
+          <t>DeepSeek V4.1 Flash</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>PITCH</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2663,12 +3029,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>GLM-5.3</t>
+          <t>DeepSeek V4.1 Flash</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>PITCH</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2691,12 +3057,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>GLM-5.3</t>
+          <t>DeepSeek V4.1 Flash</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>PITCH</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2724,7 +3090,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2752,7 +3118,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2780,7 +3146,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2808,7 +3174,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2836,7 +3202,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2864,7 +3230,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2892,7 +3258,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2920,7 +3286,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2948,7 +3314,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2976,7 +3342,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3004,7 +3370,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3032,7 +3398,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3060,7 +3426,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -3088,7 +3454,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -3116,7 +3482,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3144,7 +3510,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -3172,7 +3538,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -3200,7 +3566,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -3223,12 +3589,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Gemini-3.1-pro-preview</t>
+          <t>GLM-5.3</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -3241,22 +3607,22 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F56" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Gemini-3.1-pro-preview</t>
+          <t>GLM-5.3</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3269,22 +3635,22 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F57" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Gemini-3.1-pro-preview</t>
+          <t>GLM-5.3</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3297,59 +3663,59 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F58" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Gemini-3.1-pro-preview</t>
+          <t>GLM-5.3</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>CITE-seq CD45RA</t>
+          <t>CosMx Ki-67</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F59" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Gemini-3.1-pro-preview</t>
+          <t>GLM-5.3</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>CITE-seq CD45RA</t>
+          <t>CosMx Ki-67</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -3363,124 +3729,124 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Gemini-3.1-pro-preview</t>
+          <t>GLM-5.3</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>CITE-seq CD45RA</t>
+          <t>CosMx Ki-67</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F61" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Gemini-3.1-pro-preview</t>
+          <t>GLM-5.3</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>CITE-seq CD45RA</t>
+          <t>Gouwens input resistance</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F62" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Gemini-3.1-pro-preview</t>
+          <t>GLM-5.3</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>CITE-seq CD45RA</t>
+          <t>Gouwens input resistance</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Gemini-3.1-pro-preview</t>
+          <t>GLM-5.3</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Measurement-only</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>CITE-seq CD45RA</t>
+          <t>Gouwens input resistance</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Gemini-3.1-pro-preview</t>
+          <t>GLM-5.3</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>PITCH</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3489,26 +3855,26 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Gemini-3.1-pro-preview</t>
+          <t>GLM-5.3</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>PITCH</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3517,26 +3883,26 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F66" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Gemini-3.1-pro-preview</t>
+          <t>GLM-5.3</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>PITCH</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3545,183 +3911,183 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F67" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Gemini-3.1-pro-preview</t>
+          <t>GLM-5.3</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>PITCH</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>CITE-seq CD45RA</t>
+          <t>CosMx Ki-67</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F68" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Gemini-3.1-pro-preview</t>
+          <t>GLM-5.3</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>PITCH</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>CITE-seq CD45RA</t>
+          <t>CosMx Ki-67</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F69" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Gemini-3.1-pro-preview</t>
+          <t>GLM-5.3</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>PITCH</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>CITE-seq CD45RA</t>
+          <t>CosMx Ki-67</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F70" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Gemini-3.1-pro-preview</t>
+          <t>GLM-5.3</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>PITCH</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>CITE-seq CD45RA</t>
+          <t>Gouwens input resistance</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F71" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Gemini-3.1-pro-preview</t>
+          <t>GLM-5.3</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>PITCH</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>CITE-seq CD45RA</t>
+          <t>Gouwens input resistance</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F72" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Gemini-3.1-pro-preview</t>
+          <t>GLM-5.3</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>PITCH</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>CITE-seq CD45RA</t>
+          <t>Gouwens input resistance</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F73" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74">
@@ -3732,7 +4098,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3741,15 +4107,15 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75">
@@ -3760,7 +4126,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3769,15 +4135,15 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76">
@@ -3788,7 +4154,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3797,15 +4163,15 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F76" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77">
@@ -3816,24 +4182,24 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>CITE-seq CD45RA</t>
+          <t>CosMx Ki-67</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F77" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78">
@@ -3844,24 +4210,24 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>CITE-seq CD45RA</t>
+          <t>CosMx Ki-67</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F78" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79">
@@ -3872,24 +4238,24 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>CITE-seq CD45RA</t>
+          <t>CosMx Ki-67</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F79" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80">
@@ -3900,24 +4266,24 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>CITE-seq CD45RA</t>
+          <t>Gouwens input resistance</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F80" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81">
@@ -3928,24 +4294,24 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>CITE-seq CD45RA</t>
+          <t>Gouwens input resistance</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F81" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82">
@@ -3956,24 +4322,24 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>MLP + IG</t>
+          <t>Context-only</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>CITE-seq CD45RA</t>
+          <t>Gouwens input resistance</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F82" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83">
@@ -3993,7 +4359,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -4021,7 +4387,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -4049,7 +4415,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -4073,19 +4439,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>CosMx Ki-67</t>
+          <t>CITE-seq CD45RA</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F86" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="87">
@@ -4101,11 +4467,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>CosMx Ki-67</t>
+          <t>CITE-seq CD45RA</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -4129,11 +4495,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>CosMx Ki-67</t>
+          <t>CITE-seq CD45RA</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -4157,11 +4523,11 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>CosMx Ki-67</t>
+          <t>CITE-seq CD45RA</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -4185,11 +4551,11 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>CosMx Ki-67</t>
+          <t>CITE-seq CD45RA</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -4213,11 +4579,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>CosMx Ki-67</t>
+          <t>CITE-seq CD45RA</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -4241,19 +4607,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>CosMx Ki-67</t>
+          <t>CITE-seq CD45RA</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F92" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93">
@@ -4269,19 +4635,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Gouwens input resistance</t>
+          <t>CITE-seq CD45RA</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F93" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94">
@@ -4297,11 +4663,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Gouwens input resistance</t>
+          <t>CITE-seq CD45RA</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -4325,19 +4691,19 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Gouwens input resistance</t>
+          <t>CITE-seq CD45RA</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F95" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">
@@ -4353,19 +4719,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Gouwens input resistance</t>
+          <t>CITE-seq CD45RA</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F96" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97">
@@ -4376,7 +4742,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -4385,7 +4751,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -4404,7 +4770,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -4413,7 +4779,7 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -4432,7 +4798,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -4441,7 +4807,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -4460,16 +4826,16 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>CosMx Ki-67</t>
+          <t>CITE-seq CD45RA</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -4488,16 +4854,16 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>CosMx Ki-67</t>
+          <t>CITE-seq CD45RA</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -4516,16 +4882,16 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>CosMx Ki-67</t>
+          <t>CITE-seq CD45RA</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -4544,16 +4910,16 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Gouwens input resistance</t>
+          <t>CITE-seq CD45RA</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -4572,20 +4938,20 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Gouwens input resistance</t>
+          <t>CITE-seq CD45RA</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F104" t="b">
@@ -4600,24 +4966,24 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Measurement-only</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Gouwens input resistance</t>
+          <t>CITE-seq CD45RA</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F105" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106">
@@ -4628,7 +4994,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -4637,15 +5003,15 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F106" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="107">
@@ -4656,7 +5022,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -4665,15 +5031,15 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F107" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108">
@@ -4684,7 +5050,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -4693,15 +5059,15 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F108" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109">
@@ -4712,24 +5078,24 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>CosMx Ki-67</t>
+          <t>CITE-seq CD45RA</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F109" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110">
@@ -4740,24 +5106,24 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>CosMx Ki-67</t>
+          <t>CITE-seq CD45RA</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F110" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="111">
@@ -4768,24 +5134,24 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>CosMx Ki-67</t>
+          <t>CITE-seq CD45RA</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F111" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="112">
@@ -4796,24 +5162,24 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Gouwens input resistance</t>
+          <t>CITE-seq CD45RA</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F112" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113">
@@ -4824,16 +5190,16 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Gouwens input resistance</t>
+          <t>CosMx Ki-67</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -4852,16 +5218,16 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>PITCH</t>
+          <t>MLP + IG</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Gouwens input resistance</t>
+          <t>CosMx Ki-67</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -4875,7 +5241,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -4885,25 +5251,25 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>CITE-seq CD45RA</t>
+          <t>CosMx Ki-67</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="F115" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -4913,25 +5279,25 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>CITE-seq CD45RA</t>
+          <t>CosMx Ki-67</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F116" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -4941,25 +5307,25 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>CITE-seq CD45RA</t>
+          <t>CosMx Ki-67</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F117" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -4973,21 +5339,21 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F118" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -5001,7 +5367,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -5015,7 +5381,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -5025,11 +5391,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>CosMx Ki-67</t>
+          <t>Gouwens input resistance</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -5043,7 +5409,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -5057,21 +5423,21 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F121" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -5085,7 +5451,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -5099,7 +5465,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -5113,7 +5479,7 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -5127,7 +5493,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -5145,17 +5511,17 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F124" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -5173,7 +5539,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F125" t="b">
@@ -5183,7 +5549,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -5201,7 +5567,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F126" t="b">
@@ -5211,7 +5577,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -5229,17 +5595,17 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F127" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -5257,17 +5623,17 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F128" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -5285,17 +5651,17 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F129" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -5313,7 +5679,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>declined</t>
         </is>
       </c>
       <c r="F130" t="b">
@@ -5323,7 +5689,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -5341,7 +5707,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>declined</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="F131" t="b">
@@ -5351,7 +5717,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -5369,17 +5735,17 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>stated</t>
         </is>
       </c>
       <c r="F132" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -5407,7 +5773,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -5435,7 +5801,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -5463,7 +5829,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -5491,7 +5857,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -5519,7 +5885,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -5547,7 +5913,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -5575,7 +5941,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Qwen3.8-2.4T-A95B</t>
+          <t>Gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -5603,28 +5969,1036 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
+          <t>Gemini-3.1-pro-preview</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Gouwens input resistance</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>3</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F141" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
           <t>Qwen3.8-2.4T-A95B</t>
         </is>
       </c>
-      <c r="B141" t="inlineStr">
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Context-only</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>CITE-seq CD45RA</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>1</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F142" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Context-only</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>CITE-seq CD45RA</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>2</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F143" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Context-only</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>CITE-seq CD45RA</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>3</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F144" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Context-only</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>CosMx Ki-67</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>1</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F145" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Context-only</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>CosMx Ki-67</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>2</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F146" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Context-only</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>CosMx Ki-67</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>3</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F147" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Context-only</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Gouwens input resistance</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>1</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F148" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Context-only</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Gouwens input resistance</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>2</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F149" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Context-only</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Gouwens input resistance</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>3</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F150" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>MLP + IG</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>CITE-seq CD45RA</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>1</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F151" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>MLP + IG</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>CITE-seq CD45RA</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>2</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F152" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>MLP + IG</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>CITE-seq CD45RA</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>3</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F153" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>MLP + IG</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>CosMx Ki-67</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>1</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F154" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>MLP + IG</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>CosMx Ki-67</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>2</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F155" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>MLP + IG</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>CosMx Ki-67</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>3</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F156" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>MLP + IG</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Gouwens input resistance</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>1</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F157" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>MLP + IG</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Gouwens input resistance</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>2</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F158" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>MLP + IG</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Gouwens input resistance</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>3</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F159" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Measurement-only</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>CITE-seq CD45RA</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>1</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F160" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Measurement-only</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>CITE-seq CD45RA</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>2</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="F161" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Measurement-only</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>CITE-seq CD45RA</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>3</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="F162" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Measurement-only</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>CosMx Ki-67</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>1</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F163" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Measurement-only</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>CosMx Ki-67</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>2</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F164" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Measurement-only</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>CosMx Ki-67</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>3</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F165" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Measurement-only</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Gouwens input resistance</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>1</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="F166" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Measurement-only</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Gouwens input resistance</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>2</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>declined</t>
+        </is>
+      </c>
+      <c r="F167" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Measurement-only</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Gouwens input resistance</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>3</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="F168" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
         <is>
           <t>PITCH</t>
         </is>
       </c>
-      <c r="C141" t="inlineStr">
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>CITE-seq CD45RA</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>1</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F169" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>CITE-seq CD45RA</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>2</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F170" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>CITE-seq CD45RA</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>3</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F171" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>CosMx Ki-67</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>1</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F172" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>CosMx Ki-67</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>2</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F173" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>CosMx Ki-67</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>3</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F174" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
         <is>
           <t>Gouwens input resistance</t>
         </is>
       </c>
-      <c r="D141" t="n">
-        <v>3</v>
-      </c>
-      <c r="E141" t="inlineStr">
-        <is>
-          <t>stated</t>
-        </is>
-      </c>
-      <c r="F141" t="b">
+      <c r="D175" t="n">
+        <v>1</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F175" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Gouwens input resistance</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>2</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F176" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Qwen3.8-2.4T-A95B</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Gouwens input resistance</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>3</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>stated</t>
+        </is>
+      </c>
+      <c r="F177" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>